<commit_message>
Release 1.2.9 with date-only publication dates
</commit_message>
<xml_diff>
--- a/latest-manifest-template.xlsx
+++ b/latest-manifest-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release" sheetId="1" r:id="R29441e86ea1d49d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paths" sheetId="2" r:id="R20dde4a0c9b34855"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release" sheetId="1" r:id="Rfd9be0533be54179"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paths" sheetId="2" r:id="R4c38c348ab40423a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -155,9 +155,6 @@
     <x:t xml:space="preserve">publishedAt</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">ISO-8601 timestamp with timezone</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">filename</x:t>
   </x:si>
   <x:si>
@@ -237,6 +234,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+  </x:numFmts>
   <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
@@ -299,7 +299,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="11">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -312,6 +312,7 @@
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -733,99 +734,99 @@
       <x:c r="A22" s="1" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="B22" s="5">
-        <x:v>46337.333333333336</x:v>
-      </x:c>
-      <x:c r="C22" s="1" t="s">
-        <x:v>48</x:v>
+      <x:c r="B22" s="10" t="d">
+        <x:v>2026-11-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C22" s="1" t="str">
+        <x:v>Date: YYYY-MM-DD</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="25" customHeight="1">
       <x:c r="A23" s="1" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B23" s="5" t="s">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="B23" s="5" t="s">
+      <x:c r="C23" s="1" t="s">
         <x:v>50</x:v>
-      </x:c>
-      <x:c r="C23" s="1" t="s">
-        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="25" customHeight="1">
       <x:c r="A24" s="1" t="s">
-        <x:v>52</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="B24" s="5" t="str">
         <x:v>1.2.0</x:v>
       </x:c>
       <x:c r="C24" s="1" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="25" customHeight="1">
       <x:c r="A25" s="1" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B25" s="5" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="B25" s="5" t="s">
+      <x:c r="C25" s="1" t="s">
         <x:v>55</x:v>
-      </x:c>
-      <x:c r="C25" s="1" t="s">
-        <x:v>56</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="25" customHeight="1">
       <x:c r="A26" s="1" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B26" s="5" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="B26" s="5" t="s">
+      <x:c r="C26" s="1" t="s">
         <x:v>58</x:v>
-      </x:c>
-      <x:c r="C26" s="1" t="s">
-        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="25" customHeight="1">
       <x:c r="A27" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B27" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C27" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="25" customHeight="1">
       <x:c r="A28" s="1" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B28" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C28" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="25" customHeight="1">
       <x:c r="A29" s="1" t="s">
-        <x:v>63</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B29" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C29" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="25" customHeight="1">
       <x:c r="A30" s="1" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="B30" s="5" t="s">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="B30" s="5" t="s">
+      <x:c r="C30" s="1" t="s">
         <x:v>65</x:v>
-      </x:c>
-      <x:c r="C30" s="1" t="s">
-        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="32" customHeight="1">
@@ -855,7 +856,7 @@
   <x:sheetData>
     <x:row r="2" ht="19.299999237060547">
       <x:c r="A2" s="2" t="s">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -867,10 +868,10 @@
     </x:row>
     <x:row r="4" ht="25" customHeight="1">
       <x:c r="A4" s="3" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="s">
         <x:v>68</x:v>
-      </x:c>
-      <x:c r="B4" s="3" t="s">
-        <x:v>69</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
         <x:v>3</x:v>
@@ -878,20 +879,20 @@
     </x:row>
     <x:row r="5" ht="25" customHeight="1">
       <x:c r="A5" s="6" t="s">
-        <x:v>70</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B5" s="6"/>
       <x:c r="C5" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
       <x:c r="A6" s="6" t="s">
-        <x:v>72</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B6" s="6"/>
       <x:c r="C6" s="1" t="s">
-        <x:v>73</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">

</xml_diff>